<commit_message>
Upload file to custom window folder: فحص البرنامج.xlsx
</commit_message>
<xml_diff>
--- a/electric_unit/معلومات/فحص البرنامج.xlsx
+++ b/electric_unit/معلومات/فحص البرنامج.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\ملف السيرفر\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB24CFA-1716-45FA-834B-C052F7C767CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0F2BE1-D872-4F83-8A79-F489EDC625DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="اسناد الصيانة" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="310">
   <si>
     <t>ت</t>
   </si>
@@ -863,6 +863,99 @@
   </si>
   <si>
     <t>تنزيل</t>
+  </si>
+  <si>
+    <t>حجم الملف</t>
+  </si>
+  <si>
+    <t>عدد الملفات</t>
+  </si>
+  <si>
+    <t xml:space="preserve">إدارة أقسام (التبويبات) </t>
+  </si>
+  <si>
+    <t>إضافة قسم</t>
+  </si>
+  <si>
+    <t>تعديل قسم</t>
+  </si>
+  <si>
+    <t>حذف قسم</t>
+  </si>
+  <si>
+    <t>تجربة تكرار تسلسل قسم على قسم موجود</t>
+  </si>
+  <si>
+    <t>تجربة تكرار تسلسل قسم</t>
+  </si>
+  <si>
+    <t>ظهور الأقسام في تبويبات الاتصال والمجلدات والروابط</t>
+  </si>
+  <si>
+    <t>تسلسل ظهور النافذة</t>
+  </si>
+  <si>
+    <t>شعار النافذة (الداشبورد):</t>
+  </si>
+  <si>
+    <t>حجم شعار الجانبية:</t>
+  </si>
+  <si>
+    <t>شعار القائمة الجانبية (اختياري</t>
+  </si>
+  <si>
+    <t>حجم شعار الداشبورد:</t>
+  </si>
+  <si>
+    <t>لون خلفية الإيقونة:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رمز الدخول للنافذة </t>
+  </si>
+  <si>
+    <t xml:space="preserve">إضافة شاشة رابط جديد </t>
+  </si>
+  <si>
+    <t>إضافة مجلد</t>
+  </si>
+  <si>
+    <t>إضافة تواصل</t>
+  </si>
+  <si>
+    <t>تعديل رابط</t>
+  </si>
+  <si>
+    <t>تعديل مجلد</t>
+  </si>
+  <si>
+    <t>تعديل تواصل</t>
+  </si>
+  <si>
+    <t>ترتيب تواصل</t>
+  </si>
+  <si>
+    <t>إدارة المستخدمين</t>
+  </si>
+  <si>
+    <t>البحث المباشر</t>
+  </si>
+  <si>
+    <t>اقسام</t>
+  </si>
+  <si>
+    <t>شعب</t>
+  </si>
+  <si>
+    <t>وحدات</t>
+  </si>
+  <si>
+    <t>مسح</t>
+  </si>
+  <si>
+    <t>زر التعديل</t>
+  </si>
+  <si>
+    <t>زر الحذف</t>
   </si>
 </sst>
 </file>
@@ -873,7 +966,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -881,7 +974,7 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -955,7 +1048,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -967,14 +1060,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -982,9 +1069,27 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1266,17 +1371,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M80"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
-    <col min="3" max="5" width="5.7109375" customWidth="1"/>
-    <col min="7" max="7" width="39.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="5.7109375" customWidth="1"/>
-    <col min="13" max="13" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.75" customWidth="1"/>
+    <col min="3" max="5" width="5.75" customWidth="1"/>
+    <col min="7" max="7" width="39.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="5.75" customWidth="1"/>
+    <col min="13" max="13" width="31.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1308,7 +1413,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1328,7 +1433,7 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1348,7 +1453,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1368,7 +1473,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1388,7 +1493,7 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1408,7 +1513,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1428,7 +1533,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1448,7 +1553,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1468,7 +1573,7 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1488,7 +1593,7 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1508,7 +1613,7 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1528,7 +1633,7 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1548,7 +1653,7 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1568,7 +1673,7 @@
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1588,7 +1693,7 @@
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
     </row>
-    <row r="16" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1608,7 +1713,7 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1628,7 +1733,7 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1648,7 +1753,7 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1668,7 +1773,7 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1688,7 +1793,7 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1708,7 +1813,7 @@
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
     </row>
-    <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1728,7 +1833,7 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
     </row>
-    <row r="23" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1748,7 +1853,7 @@
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
     </row>
-    <row r="24" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1768,7 +1873,7 @@
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
     </row>
-    <row r="25" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1788,7 +1893,7 @@
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
     </row>
-    <row r="26" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1808,7 +1913,7 @@
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
     </row>
-    <row r="27" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1828,7 +1933,7 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
     </row>
-    <row r="28" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1848,7 +1953,7 @@
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
     </row>
-    <row r="29" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1868,7 +1973,7 @@
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
     </row>
-    <row r="30" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1888,7 +1993,7 @@
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
     </row>
-    <row r="31" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1908,7 +2013,7 @@
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
     </row>
-    <row r="32" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1928,7 +2033,7 @@
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
     </row>
-    <row r="33" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1948,7 +2053,7 @@
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
     </row>
-    <row r="34" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1968,7 +2073,7 @@
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
     </row>
-    <row r="35" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1988,7 +2093,7 @@
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
     </row>
-    <row r="36" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -2008,7 +2113,7 @@
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
     </row>
-    <row r="37" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -2028,7 +2133,7 @@
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
     </row>
-    <row r="38" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -2048,7 +2153,7 @@
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
     </row>
-    <row r="39" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -2068,7 +2173,7 @@
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
     </row>
-    <row r="40" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -2088,7 +2193,7 @@
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
     </row>
-    <row r="41" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -2108,7 +2213,7 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -2128,7 +2233,7 @@
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
     </row>
-    <row r="43" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -2148,7 +2253,7 @@
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
     </row>
-    <row r="44" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -2168,7 +2273,7 @@
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
     </row>
-    <row r="45" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -2188,7 +2293,7 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
     </row>
-    <row r="46" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -2208,7 +2313,7 @@
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
     </row>
-    <row r="47" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -2228,7 +2333,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
     </row>
-    <row r="48" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -2248,7 +2353,7 @@
       <c r="I48" s="1"/>
       <c r="J48" s="1"/>
     </row>
-    <row r="49" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -2268,7 +2373,7 @@
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
     </row>
-    <row r="50" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -2288,7 +2393,7 @@
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
     </row>
-    <row r="51" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -2308,7 +2413,7 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
     </row>
-    <row r="52" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -2328,7 +2433,7 @@
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
     </row>
-    <row r="53" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -2348,7 +2453,7 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
     </row>
-    <row r="54" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -2368,7 +2473,7 @@
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
     </row>
-    <row r="55" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -2388,7 +2493,7 @@
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
     </row>
-    <row r="56" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -2408,7 +2513,7 @@
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
     </row>
-    <row r="57" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -2428,7 +2533,7 @@
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
     </row>
-    <row r="58" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -2448,7 +2553,7 @@
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
     </row>
-    <row r="59" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -2468,7 +2573,7 @@
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
     </row>
-    <row r="60" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -2488,7 +2593,7 @@
       <c r="I60" s="1"/>
       <c r="J60" s="1"/>
     </row>
-    <row r="61" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -2508,7 +2613,7 @@
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
     </row>
-    <row r="62" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -2528,7 +2633,7 @@
       <c r="I62" s="1"/>
       <c r="J62" s="1"/>
     </row>
-    <row r="63" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -2548,7 +2653,7 @@
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
     </row>
-    <row r="64" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -2568,7 +2673,7 @@
       <c r="I64" s="1"/>
       <c r="J64" s="1"/>
     </row>
-    <row r="65" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -2588,7 +2693,7 @@
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
     </row>
-    <row r="66" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -2608,7 +2713,7 @@
       <c r="I66" s="1"/>
       <c r="J66" s="1"/>
     </row>
-    <row r="67" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -2628,7 +2733,7 @@
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
     </row>
-    <row r="68" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -2648,7 +2753,7 @@
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
     </row>
-    <row r="69" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -2668,7 +2773,7 @@
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
     </row>
-    <row r="70" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -2688,7 +2793,7 @@
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
     </row>
-    <row r="71" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -2708,7 +2813,7 @@
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
     </row>
-    <row r="72" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -2728,7 +2833,7 @@
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
     </row>
-    <row r="73" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -2748,7 +2853,7 @@
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
     </row>
-    <row r="74" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -2766,7 +2871,7 @@
       <c r="I74" s="1"/>
       <c r="J74" s="1"/>
     </row>
-    <row r="75" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -2784,7 +2889,7 @@
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
     </row>
-    <row r="76" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -2802,19 +2907,19 @@
       <c r="I76" s="1"/>
       <c r="J76" s="1"/>
     </row>
-    <row r="80" spans="1:13" ht="186.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="5"/>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5"/>
-      <c r="E80" s="5"/>
-      <c r="F80" s="5"/>
-      <c r="G80" s="5"/>
-      <c r="H80" s="5"/>
-      <c r="I80" s="5"/>
-      <c r="J80" s="5"/>
-      <c r="K80" s="5"/>
-      <c r="L80" s="5"/>
-      <c r="M80" s="5"/>
+    <row r="80" spans="1:13" ht="186.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B80" s="8"/>
+      <c r="C80" s="8"/>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8"/>
+      <c r="G80" s="8"/>
+      <c r="H80" s="8"/>
+      <c r="I80" s="8"/>
+      <c r="J80" s="8"/>
+      <c r="K80" s="8"/>
+      <c r="L80" s="8"/>
+      <c r="M80" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2831,18 +2936,18 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M256"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
-    <col min="3" max="5" width="5.7109375" customWidth="1"/>
-    <col min="7" max="7" width="39.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="5.7109375" customWidth="1"/>
-    <col min="13" max="13" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.75" customWidth="1"/>
+    <col min="3" max="5" width="5.75" customWidth="1"/>
+    <col min="7" max="7" width="39.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="5.75" customWidth="1"/>
+    <col min="13" max="13" width="31.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2874,7 +2979,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -2894,7 +2999,7 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2914,7 +3019,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2934,7 +3039,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2954,7 +3059,7 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2974,11 +3079,11 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>154</v>
       </c>
       <c r="C7" s="1"/>
@@ -2994,7 +3099,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -3014,7 +3119,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -3033,9 +3138,9 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
-      <c r="M9" s="7"/>
-    </row>
-    <row r="10" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M9" s="9"/>
+    </row>
+    <row r="10" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -3054,9 +3159,9 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
-      <c r="M10" s="7"/>
-    </row>
-    <row r="11" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M10" s="9"/>
+    </row>
+    <row r="11" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -3075,9 +3180,9 @@
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
-      <c r="M11" s="7"/>
-    </row>
-    <row r="12" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M11" s="9"/>
+    </row>
+    <row r="12" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -3096,9 +3201,9 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="M12" s="7"/>
-    </row>
-    <row r="13" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M12" s="9"/>
+    </row>
+    <row r="13" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -3117,9 +3222,9 @@
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
-      <c r="M13" s="7"/>
-    </row>
-    <row r="14" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M13" s="9"/>
+    </row>
+    <row r="14" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -3138,9 +3243,9 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
-      <c r="M14" s="7"/>
-    </row>
-    <row r="15" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M14" s="9"/>
+    </row>
+    <row r="15" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -3159,9 +3264,9 @@
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
-      <c r="M15" s="7"/>
-    </row>
-    <row r="16" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M15" s="9"/>
+    </row>
+    <row r="16" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -3180,13 +3285,13 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
-      <c r="M16" s="7"/>
-    </row>
-    <row r="17" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M16" s="9"/>
+    </row>
+    <row r="17" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>164</v>
       </c>
       <c r="C17" s="1"/>
@@ -3202,7 +3307,7 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -3222,7 +3327,7 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -3242,7 +3347,7 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -3262,7 +3367,7 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -3282,7 +3387,7 @@
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
     </row>
-    <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -3302,7 +3407,7 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
     </row>
-    <row r="23" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -3322,7 +3427,7 @@
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
     </row>
-    <row r="24" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -3342,7 +3447,7 @@
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
     </row>
-    <row r="25" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -3362,7 +3467,7 @@
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
     </row>
-    <row r="26" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -3382,7 +3487,7 @@
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
     </row>
-    <row r="27" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -3402,7 +3507,7 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
     </row>
-    <row r="28" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -3422,7 +3527,7 @@
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
     </row>
-    <row r="29" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -3442,7 +3547,7 @@
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
     </row>
-    <row r="30" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -3462,7 +3567,7 @@
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
     </row>
-    <row r="31" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -3482,7 +3587,7 @@
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
     </row>
-    <row r="32" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -3495,14 +3600,14 @@
       <c r="F32" s="3">
         <v>68</v>
       </c>
-      <c r="G32" s="8" t="s">
+      <c r="G32" s="6" t="s">
         <v>212</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
     </row>
-    <row r="33" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -3522,7 +3627,7 @@
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
     </row>
-    <row r="34" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -3542,7 +3647,7 @@
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
     </row>
-    <row r="35" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -3562,7 +3667,7 @@
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
     </row>
-    <row r="36" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -3582,7 +3687,7 @@
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
     </row>
-    <row r="37" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -3602,7 +3707,7 @@
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
     </row>
-    <row r="38" spans="1:10" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -3622,7 +3727,7 @@
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
     </row>
-    <row r="39" spans="1:10" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>0</v>
       </c>
@@ -3654,7 +3759,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>75</v>
       </c>
@@ -3674,7 +3779,7 @@
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
     </row>
-    <row r="41" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>76</v>
       </c>
@@ -3687,14 +3792,14 @@
       <c r="F41" s="3">
         <v>114</v>
       </c>
-      <c r="G41" s="8" t="s">
+      <c r="G41" s="6" t="s">
         <v>257</v>
       </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
     </row>
-    <row r="42" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>77</v>
       </c>
@@ -3714,7 +3819,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>78</v>
       </c>
@@ -3734,7 +3839,7 @@
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
     </row>
-    <row r="44" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>79</v>
       </c>
@@ -3754,7 +3859,7 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
     </row>
-    <row r="45" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>80</v>
       </c>
@@ -3774,7 +3879,7 @@
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
     </row>
-    <row r="46" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>81</v>
       </c>
@@ -3794,7 +3899,7 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
     </row>
-    <row r="47" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>82</v>
       </c>
@@ -3814,7 +3919,7 @@
       <c r="I47" s="1"/>
       <c r="J47" s="1"/>
     </row>
-    <row r="48" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>83</v>
       </c>
@@ -3834,7 +3939,7 @@
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
     </row>
-    <row r="49" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>84</v>
       </c>
@@ -3854,11 +3959,11 @@
       <c r="I49" s="1"/>
       <c r="J49" s="1"/>
     </row>
-    <row r="50" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>85</v>
       </c>
-      <c r="B50" s="9" t="s">
+      <c r="B50" s="7" t="s">
         <v>229</v>
       </c>
       <c r="C50" s="2"/>
@@ -3874,11 +3979,11 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
     </row>
-    <row r="51" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>86</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B51" s="7" t="s">
         <v>230</v>
       </c>
       <c r="C51" s="1"/>
@@ -3887,14 +3992,14 @@
       <c r="F51" s="3">
         <v>124</v>
       </c>
-      <c r="G51" s="8" t="s">
+      <c r="G51" s="6" t="s">
         <v>266</v>
       </c>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
       <c r="J51" s="1"/>
     </row>
-    <row r="52" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>87</v>
       </c>
@@ -3914,11 +4019,11 @@
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
     </row>
-    <row r="53" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>88</v>
       </c>
-      <c r="B53" s="9" t="s">
+      <c r="B53" s="7" t="s">
         <v>232</v>
       </c>
       <c r="C53" s="1"/>
@@ -3934,7 +4039,7 @@
       <c r="I53" s="1"/>
       <c r="J53" s="1"/>
     </row>
-    <row r="54" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>89</v>
       </c>
@@ -3954,7 +4059,7 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
     </row>
-    <row r="55" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>90</v>
       </c>
@@ -3974,7 +4079,7 @@
       <c r="I55" s="1"/>
       <c r="J55" s="1"/>
     </row>
-    <row r="56" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>91</v>
       </c>
@@ -3994,7 +4099,7 @@
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
     </row>
-    <row r="57" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>92</v>
       </c>
@@ -4014,7 +4119,7 @@
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
     </row>
-    <row r="58" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>93</v>
       </c>
@@ -4034,7 +4139,7 @@
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
     </row>
-    <row r="59" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>94</v>
       </c>
@@ -4054,7 +4159,7 @@
       <c r="I59" s="1"/>
       <c r="J59" s="1"/>
     </row>
-    <row r="60" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>95</v>
       </c>
@@ -4074,7 +4179,7 @@
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
     </row>
-    <row r="61" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>96</v>
       </c>
@@ -4094,7 +4199,7 @@
       <c r="I61" s="1"/>
       <c r="J61" s="1"/>
     </row>
-    <row r="62" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>97</v>
       </c>
@@ -4114,7 +4219,7 @@
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
     </row>
-    <row r="63" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>98</v>
       </c>
@@ -4134,7 +4239,7 @@
       <c r="I63" s="1"/>
       <c r="J63" s="1"/>
     </row>
-    <row r="64" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>99</v>
       </c>
@@ -4147,12 +4252,14 @@
       <c r="F64" s="1">
         <v>137</v>
       </c>
-      <c r="G64" s="3"/>
+      <c r="G64" s="3" t="s">
+        <v>279</v>
+      </c>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
     </row>
-    <row r="65" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>100</v>
       </c>
@@ -4165,12 +4272,14 @@
       <c r="F65" s="3">
         <v>138</v>
       </c>
-      <c r="G65" s="3"/>
+      <c r="G65" s="3" t="s">
+        <v>280</v>
+      </c>
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
       <c r="J65" s="1"/>
     </row>
-    <row r="66" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>101</v>
       </c>
@@ -4183,12 +4292,14 @@
       <c r="F66" s="1">
         <v>139</v>
       </c>
-      <c r="G66" s="3"/>
+      <c r="G66" s="3" t="s">
+        <v>281</v>
+      </c>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
     </row>
-    <row r="67" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>102</v>
       </c>
@@ -4201,12 +4312,14 @@
       <c r="F67" s="3">
         <v>140</v>
       </c>
-      <c r="G67" s="3"/>
+      <c r="G67" s="3" t="s">
+        <v>282</v>
+      </c>
       <c r="H67" s="1"/>
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
     </row>
-    <row r="68" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>103</v>
       </c>
@@ -4219,12 +4332,14 @@
       <c r="F68" s="1">
         <v>141</v>
       </c>
-      <c r="G68" s="3"/>
+      <c r="G68" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
     </row>
-    <row r="69" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>104</v>
       </c>
@@ -4237,16 +4352,18 @@
       <c r="F69" s="3">
         <v>142</v>
       </c>
-      <c r="G69" s="3"/>
+      <c r="G69" s="3" t="s">
+        <v>284</v>
+      </c>
       <c r="H69" s="1"/>
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
     </row>
-    <row r="70" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>105</v>
       </c>
-      <c r="B70" s="6" t="s">
+      <c r="B70" s="5" t="s">
         <v>248</v>
       </c>
       <c r="C70" s="2"/>
@@ -4255,12 +4372,14 @@
       <c r="F70" s="1">
         <v>143</v>
       </c>
-      <c r="G70" s="3"/>
+      <c r="G70" s="3" t="s">
+        <v>286</v>
+      </c>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
     </row>
-    <row r="71" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>106</v>
       </c>
@@ -4273,12 +4392,14 @@
       <c r="F71" s="3">
         <v>144</v>
       </c>
-      <c r="G71" s="3"/>
+      <c r="G71" s="3" t="s">
+        <v>285</v>
+      </c>
       <c r="H71" s="1"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
     </row>
-    <row r="72" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>107</v>
       </c>
@@ -4291,12 +4412,14 @@
       <c r="F72" s="1">
         <v>145</v>
       </c>
-      <c r="G72" s="3"/>
+      <c r="G72" s="3" t="s">
+        <v>287</v>
+      </c>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
     </row>
-    <row r="73" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>108</v>
       </c>
@@ -4309,12 +4432,14 @@
       <c r="F73" s="3">
         <v>146</v>
       </c>
-      <c r="G73" s="3"/>
+      <c r="G73" s="3" t="s">
+        <v>288</v>
+      </c>
       <c r="H73" s="1"/>
       <c r="I73" s="1"/>
       <c r="J73" s="1"/>
     </row>
-    <row r="74" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>109</v>
       </c>
@@ -4327,12 +4452,14 @@
       <c r="F74" s="1">
         <v>147</v>
       </c>
-      <c r="G74" s="3"/>
+      <c r="G74" s="3" t="s">
+        <v>214</v>
+      </c>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
     </row>
-    <row r="75" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>110</v>
       </c>
@@ -4345,12 +4472,14 @@
       <c r="F75" s="3">
         <v>148</v>
       </c>
-      <c r="G75" s="3"/>
+      <c r="G75" s="3" t="s">
+        <v>215</v>
+      </c>
       <c r="H75" s="1"/>
       <c r="I75" s="1"/>
       <c r="J75" s="1"/>
     </row>
-    <row r="76" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>111</v>
       </c>
@@ -4363,12 +4492,14 @@
       <c r="F76" s="1">
         <v>149</v>
       </c>
-      <c r="G76" s="3"/>
+      <c r="G76" s="3" t="s">
+        <v>216</v>
+      </c>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
     </row>
-    <row r="77" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>112</v>
       </c>
@@ -4381,28 +4512,842 @@
       <c r="F77" s="3">
         <v>150</v>
       </c>
-      <c r="G77" s="3"/>
+      <c r="G77" s="3" t="s">
+        <v>289</v>
+      </c>
       <c r="H77" s="1"/>
       <c r="I77" s="1"/>
       <c r="J77" s="1"/>
     </row>
-    <row r="81" spans="2:13" ht="186.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="5"/>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="5"/>
-      <c r="G81" s="5"/>
-      <c r="H81" s="5"/>
-      <c r="I81" s="5"/>
-      <c r="J81" s="5"/>
-      <c r="K81" s="5"/>
-      <c r="L81" s="5"/>
-      <c r="M81" s="5"/>
-    </row>
+    <row r="78" spans="1:10" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F78" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G78" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H78" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I78" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J78" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="1">
+        <v>151</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C79" s="1"/>
+      <c r="D79" s="1"/>
+      <c r="E79" s="1"/>
+      <c r="F79" s="1">
+        <v>189</v>
+      </c>
+      <c r="G79" s="3"/>
+      <c r="H79" s="1"/>
+      <c r="I79" s="1"/>
+      <c r="J79" s="1"/>
+    </row>
+    <row r="80" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="1">
+        <v>152</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C80" s="1"/>
+      <c r="D80" s="1"/>
+      <c r="E80" s="1"/>
+      <c r="F80" s="3">
+        <v>190</v>
+      </c>
+      <c r="G80" s="12"/>
+      <c r="H80" s="1"/>
+      <c r="I80" s="1"/>
+      <c r="J80" s="1"/>
+    </row>
+    <row r="81" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="1">
+        <v>153</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2"/>
+      <c r="F81" s="1">
+        <v>191</v>
+      </c>
+      <c r="G81" s="12"/>
+      <c r="H81" s="2"/>
+      <c r="I81" s="2"/>
+      <c r="J81" s="2"/>
+      <c r="K81" s="10"/>
+      <c r="L81" s="10"/>
+      <c r="M81" s="10"/>
+    </row>
+    <row r="82" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="1">
+        <v>154</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C82" s="1"/>
+      <c r="D82" s="1"/>
+      <c r="E82" s="1"/>
+      <c r="F82" s="3">
+        <v>192</v>
+      </c>
+      <c r="G82" s="12"/>
+      <c r="H82" s="1"/>
+      <c r="I82" s="1"/>
+      <c r="J82" s="1"/>
+    </row>
+    <row r="83" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="1">
+        <v>155</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2"/>
+      <c r="F83" s="1">
+        <v>193</v>
+      </c>
+      <c r="G83" s="12"/>
+      <c r="H83" s="2"/>
+      <c r="I83" s="2"/>
+      <c r="J83" s="2"/>
+    </row>
+    <row r="84" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="1">
+        <v>156</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C84" s="1"/>
+      <c r="D84" s="1"/>
+      <c r="E84" s="1"/>
+      <c r="F84" s="3">
+        <v>194</v>
+      </c>
+      <c r="G84" s="12"/>
+      <c r="H84" s="1"/>
+      <c r="I84" s="1"/>
+      <c r="J84" s="1"/>
+    </row>
+    <row r="85" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="1">
+        <v>157</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C85" s="2"/>
+      <c r="D85" s="2"/>
+      <c r="E85" s="2"/>
+      <c r="F85" s="1">
+        <v>195</v>
+      </c>
+      <c r="G85" s="12"/>
+      <c r="H85" s="2"/>
+      <c r="I85" s="2"/>
+      <c r="J85" s="2"/>
+    </row>
+    <row r="86" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="1">
+        <v>158</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+      <c r="F86" s="3">
+        <v>196</v>
+      </c>
+      <c r="G86" s="12"/>
+      <c r="H86" s="1"/>
+      <c r="I86" s="1"/>
+      <c r="J86" s="1"/>
+    </row>
+    <row r="87" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="1">
+        <v>159</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
+      <c r="E87" s="2"/>
+      <c r="F87" s="1">
+        <v>197</v>
+      </c>
+      <c r="G87" s="12"/>
+      <c r="H87" s="2"/>
+      <c r="I87" s="2"/>
+      <c r="J87" s="2"/>
+    </row>
+    <row r="88" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="1">
+        <v>160</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+      <c r="F88" s="3">
+        <v>198</v>
+      </c>
+      <c r="G88" s="12"/>
+      <c r="H88" s="1"/>
+      <c r="I88" s="1"/>
+      <c r="J88" s="1"/>
+    </row>
+    <row r="89" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="1">
+        <v>161</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="1">
+        <v>199</v>
+      </c>
+      <c r="G89" s="12"/>
+      <c r="H89" s="2"/>
+      <c r="I89" s="2"/>
+      <c r="J89" s="2"/>
+    </row>
+    <row r="90" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="1">
+        <v>162</v>
+      </c>
+      <c r="B90" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="3">
+        <v>200</v>
+      </c>
+      <c r="G90" s="12"/>
+      <c r="H90" s="1"/>
+      <c r="I90" s="1"/>
+      <c r="J90" s="1"/>
+    </row>
+    <row r="91" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="1">
+        <v>163</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="E91" s="2"/>
+      <c r="F91" s="1">
+        <v>201</v>
+      </c>
+      <c r="G91" s="12"/>
+      <c r="H91" s="2"/>
+      <c r="I91" s="2"/>
+      <c r="J91" s="2"/>
+    </row>
+    <row r="92" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" s="1">
+        <v>164</v>
+      </c>
+      <c r="B92" s="13" t="s">
+        <v>302</v>
+      </c>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+      <c r="F92" s="3">
+        <v>202</v>
+      </c>
+      <c r="G92" s="12"/>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1"/>
+      <c r="J92" s="1"/>
+    </row>
+    <row r="93" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A93" s="1">
+        <v>165</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="E93" s="2"/>
+      <c r="F93" s="1">
+        <v>203</v>
+      </c>
+      <c r="G93" s="3"/>
+      <c r="H93" s="2"/>
+      <c r="I93" s="2"/>
+      <c r="J93" s="2"/>
+    </row>
+    <row r="94" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="1">
+        <v>166</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="3">
+        <v>204</v>
+      </c>
+      <c r="G94" s="3"/>
+      <c r="H94" s="1"/>
+      <c r="I94" s="1"/>
+      <c r="J94" s="1"/>
+    </row>
+    <row r="95" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="1">
+        <v>167</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C95" s="2"/>
+      <c r="D95" s="2"/>
+      <c r="E95" s="2"/>
+      <c r="F95" s="1">
+        <v>205</v>
+      </c>
+      <c r="G95" s="3"/>
+      <c r="H95" s="2"/>
+      <c r="I95" s="2"/>
+      <c r="J95" s="2"/>
+    </row>
+    <row r="96" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="1">
+        <v>168</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="3">
+        <v>206</v>
+      </c>
+      <c r="G96" s="3"/>
+      <c r="H96" s="1"/>
+      <c r="I96" s="1"/>
+      <c r="J96" s="1"/>
+    </row>
+    <row r="97" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" s="1">
+        <v>169</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2"/>
+      <c r="E97" s="2"/>
+      <c r="F97" s="1">
+        <v>207</v>
+      </c>
+      <c r="G97" s="3"/>
+      <c r="H97" s="2"/>
+      <c r="I97" s="2"/>
+      <c r="J97" s="2"/>
+    </row>
+    <row r="98" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A98" s="1">
+        <v>170</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C98" s="1"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="F98" s="3">
+        <v>208</v>
+      </c>
+      <c r="G98" s="3"/>
+      <c r="H98" s="1"/>
+      <c r="I98" s="1"/>
+      <c r="J98" s="1"/>
+    </row>
+    <row r="99" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="1">
+        <v>171</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+      <c r="E99" s="2"/>
+      <c r="F99" s="1">
+        <v>209</v>
+      </c>
+      <c r="G99" s="3"/>
+      <c r="H99" s="2"/>
+      <c r="I99" s="2"/>
+      <c r="J99" s="2"/>
+    </row>
+    <row r="100" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="1">
+        <v>172</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="F100" s="3">
+        <v>210</v>
+      </c>
+      <c r="G100" s="3"/>
+      <c r="H100" s="1"/>
+      <c r="I100" s="1"/>
+      <c r="J100" s="1"/>
+    </row>
+    <row r="101" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A101" s="1">
+        <v>173</v>
+      </c>
+      <c r="B101" s="1"/>
+      <c r="C101" s="2"/>
+      <c r="D101" s="2"/>
+      <c r="E101" s="2"/>
+      <c r="F101" s="1">
+        <v>211</v>
+      </c>
+      <c r="G101" s="3"/>
+      <c r="H101" s="2"/>
+      <c r="I101" s="2"/>
+      <c r="J101" s="2"/>
+    </row>
+    <row r="102" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A102" s="1">
+        <v>174</v>
+      </c>
+      <c r="B102" s="1"/>
+      <c r="C102" s="1"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="F102" s="3">
+        <v>212</v>
+      </c>
+      <c r="G102" s="3"/>
+      <c r="H102" s="1"/>
+      <c r="I102" s="1"/>
+      <c r="J102" s="1"/>
+    </row>
+    <row r="103" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A103" s="1">
+        <v>175</v>
+      </c>
+      <c r="B103" s="1"/>
+      <c r="C103" s="2"/>
+      <c r="D103" s="2"/>
+      <c r="E103" s="2"/>
+      <c r="F103" s="1">
+        <v>213</v>
+      </c>
+      <c r="G103" s="3"/>
+      <c r="H103" s="2"/>
+      <c r="I103" s="2"/>
+      <c r="J103" s="2"/>
+    </row>
+    <row r="104" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A104" s="1">
+        <v>176</v>
+      </c>
+      <c r="B104" s="1"/>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="3">
+        <v>214</v>
+      </c>
+      <c r="G104" s="3"/>
+      <c r="H104" s="1"/>
+      <c r="I104" s="1"/>
+      <c r="J104" s="1"/>
+    </row>
+    <row r="105" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A105" s="1">
+        <v>177</v>
+      </c>
+      <c r="B105" s="1"/>
+      <c r="C105" s="2"/>
+      <c r="D105" s="2"/>
+      <c r="E105" s="2"/>
+      <c r="F105" s="1">
+        <v>215</v>
+      </c>
+      <c r="G105" s="3"/>
+      <c r="H105" s="2"/>
+      <c r="I105" s="2"/>
+      <c r="J105" s="2"/>
+    </row>
+    <row r="106" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="1">
+        <v>178</v>
+      </c>
+      <c r="B106" s="1"/>
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
+      <c r="F106" s="3">
+        <v>216</v>
+      </c>
+      <c r="G106" s="3"/>
+      <c r="H106" s="1"/>
+      <c r="I106" s="1"/>
+      <c r="J106" s="1"/>
+    </row>
+    <row r="107" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A107" s="1">
+        <v>179</v>
+      </c>
+      <c r="B107" s="11"/>
+      <c r="C107" s="2"/>
+      <c r="D107" s="2"/>
+      <c r="E107" s="2"/>
+      <c r="F107" s="1">
+        <v>217</v>
+      </c>
+      <c r="G107" s="3"/>
+      <c r="H107" s="2"/>
+      <c r="I107" s="2"/>
+      <c r="J107" s="2"/>
+    </row>
+    <row r="108" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A108" s="1">
+        <v>180</v>
+      </c>
+      <c r="B108" s="12"/>
+      <c r="C108" s="1"/>
+      <c r="D108" s="1"/>
+      <c r="E108" s="1"/>
+      <c r="F108" s="3">
+        <v>218</v>
+      </c>
+      <c r="G108" s="3"/>
+      <c r="H108" s="1"/>
+      <c r="I108" s="1"/>
+      <c r="J108" s="1"/>
+    </row>
+    <row r="109" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A109" s="1">
+        <v>181</v>
+      </c>
+      <c r="B109" s="11"/>
+      <c r="C109" s="2"/>
+      <c r="D109" s="2"/>
+      <c r="E109" s="2"/>
+      <c r="F109" s="1">
+        <v>219</v>
+      </c>
+      <c r="G109" s="3"/>
+      <c r="H109" s="2"/>
+      <c r="I109" s="2"/>
+      <c r="J109" s="2"/>
+    </row>
+    <row r="110" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A110" s="1">
+        <v>182</v>
+      </c>
+      <c r="B110" s="11"/>
+      <c r="C110" s="1"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+      <c r="F110" s="3">
+        <v>220</v>
+      </c>
+      <c r="G110" s="3"/>
+      <c r="H110" s="1"/>
+      <c r="I110" s="1"/>
+      <c r="J110" s="1"/>
+    </row>
+    <row r="111" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A111" s="1">
+        <v>183</v>
+      </c>
+      <c r="B111" s="11"/>
+      <c r="C111" s="2"/>
+      <c r="D111" s="2"/>
+      <c r="E111" s="2"/>
+      <c r="F111" s="1">
+        <v>221</v>
+      </c>
+      <c r="G111" s="3"/>
+      <c r="H111" s="2"/>
+      <c r="I111" s="2"/>
+      <c r="J111" s="2"/>
+    </row>
+    <row r="112" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A112" s="1">
+        <v>184</v>
+      </c>
+      <c r="B112" s="1"/>
+      <c r="C112" s="1"/>
+      <c r="D112" s="1"/>
+      <c r="E112" s="1"/>
+      <c r="F112" s="3">
+        <v>222</v>
+      </c>
+      <c r="G112" s="3"/>
+      <c r="H112" s="1"/>
+      <c r="I112" s="1"/>
+      <c r="J112" s="1"/>
+    </row>
+    <row r="113" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="1">
+        <v>185</v>
+      </c>
+      <c r="B113" s="1"/>
+      <c r="C113" s="2"/>
+      <c r="D113" s="2"/>
+      <c r="E113" s="2"/>
+      <c r="F113" s="1">
+        <v>223</v>
+      </c>
+      <c r="G113" s="3"/>
+      <c r="H113" s="2"/>
+      <c r="I113" s="2"/>
+      <c r="J113" s="2"/>
+    </row>
+    <row r="114" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A114" s="1">
+        <v>186</v>
+      </c>
+      <c r="B114" s="1"/>
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="1"/>
+      <c r="F114" s="3">
+        <v>224</v>
+      </c>
+      <c r="G114" s="3"/>
+      <c r="H114" s="1"/>
+      <c r="I114" s="1"/>
+      <c r="J114" s="1"/>
+    </row>
+    <row r="115" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A115" s="1">
+        <v>187</v>
+      </c>
+      <c r="B115" s="1"/>
+      <c r="C115" s="2"/>
+      <c r="D115" s="2"/>
+      <c r="E115" s="2"/>
+      <c r="F115" s="1">
+        <v>225</v>
+      </c>
+      <c r="G115" s="3"/>
+      <c r="H115" s="2"/>
+      <c r="I115" s="2"/>
+      <c r="J115" s="2"/>
+    </row>
+    <row r="116" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A116" s="1">
+        <v>188</v>
+      </c>
+      <c r="B116" s="1"/>
+      <c r="C116" s="1"/>
+      <c r="D116" s="1"/>
+      <c r="E116" s="1"/>
+      <c r="F116" s="3">
+        <v>226</v>
+      </c>
+      <c r="G116" s="3"/>
+      <c r="H116" s="1"/>
+      <c r="I116" s="1"/>
+      <c r="J116" s="1"/>
+    </row>
+    <row r="117" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="118" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="119" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="120" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="121" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="122" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="123" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="124" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="125" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="126" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="127" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="128" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="129" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="130" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="131" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="132" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="133" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="134" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="135" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="136" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="137" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="138" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="139" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="140" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="141" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="142" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="143" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="144" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="145" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="146" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="147" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="148" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="149" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="150" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="151" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="152" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="153" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="154" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="155" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="156" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="157" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="158" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="159" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="160" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="161" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="162" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="163" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="164" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="165" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="166" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="167" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="168" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="169" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="170" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="171" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="172" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="173" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="174" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="175" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="176" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="177" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="178" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="179" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="180" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="181" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="182" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="183" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="184" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="185" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="186" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="187" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="188" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="189" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="190" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="191" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="192" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="193" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="194" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="195" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="196" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="197" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="198" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="199" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="200" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="201" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="202" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="203" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="204" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="205" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="206" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="207" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="208" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="209" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="210" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="211" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="212" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="213" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="214" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="215" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="216" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="217" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="218" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="219" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="220" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="221" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="222" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="223" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="224" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="225" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="226" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="227" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="228" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="229" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="230" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="231" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="232" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="233" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="234" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="235" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="236" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="237" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="238" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="239" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="240" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="241" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="242" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="243" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="244" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="245" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="246" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="247" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="248" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="249" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="250" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="251" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="252" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="253" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="254" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="255" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="256" ht="24.95" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B81:M81"/>
+  <mergeCells count="1">
     <mergeCell ref="M9:M16"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>